<commit_message>
## Filter Tanggal Ditambahkan
- **Dashboard & Laporan** kini memiliki filter periode: Hari ini · Minggu ini · Bulan ini · Tahun ini · Kustom (2 date-picker)
- KPI **Omzet Periode**, **Laba Kotor**, dan **Top Penjualan** ikut berubah mengikuti rentang yang dipilih; chart bar dinamis merangkai omzet per hari dalam rentang
- Endpoint diperluas: `GET /api/dashboard?start=&end=` & `GET /api/sales?start=&end=` — diverifikasi via curl (rentang harian, bulanan, kustom semua benar)

- Next Action Items:
  - **Detail Produk**: Buka halaman detail penuh dengan grafik penjualan dan histori barang masuk per SKU
  - **Cetak Invoice**: Beri tombol cetak PDF dari halaman Penjualan sehingga bisa langsung dikirim ke customer
  - **Retur Penjualan**: Tambah alur retur yang otomatis mengoreksi stok dan omzet
  - **Filter Produk & Kategori**: Perluas filter Laporan agar bisa disaring per SKU, brand, atau kategori
</commit_message>
<xml_diff>
--- a/backend/inventory.xlsx
+++ b/backend/inventory.xlsx
@@ -526,10 +526,8 @@
           <t>MTC-300</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>899100300001</t>
-        </is>
+      <c r="C2" t="n">
+        <v>899100300001</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -571,7 +569,7 @@
         <v>6800000</v>
       </c>
       <c r="M2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N2" t="n">
         <v>3</v>
@@ -596,7 +594,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-09-04T07:08:55.442424+00:00</t>
+          <t>2026-09-04T07:14:20.249676+00:00</t>
         </is>
       </c>
     </row>
@@ -611,10 +609,8 @@
           <t>KTN-87A05</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>899100300002</t>
-        </is>
+      <c r="C3" t="n">
+        <v>899100300002</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -696,10 +692,8 @@
           <t>INS-2301-10</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>899100300003</t>
-        </is>
+      <c r="C4" t="n">
+        <v>899100300003</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -781,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1076,6 +1070,120 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1de3f46f-963e-454d-a663-8b4db37bd86b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GR-960473</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MTC-300</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tire Charger</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Barang Masuk</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>on stocl</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:14:19.384855+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>18ce311c-f924-4d8f-add0-fa12ed7e08fc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GR-960473</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MTC-300</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tire Charger</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Barang Masuk</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>11</v>
+      </c>
+      <c r="I7" t="n">
+        <v>12</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>on stocl</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:14:20.249676+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>